<commit_message>
files are modified and push
</commit_message>
<xml_diff>
--- a/data/excel/TestData.xlsx
+++ b/data/excel/TestData.xlsx
@@ -1,49 +1,115 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" r:id="rId2"/>
-    <sheet name="ForgotPassword" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Login" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Dashboard" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="ForgotPassword" state="visible" r:id="rId6"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>EMIS | Tamil Nadu Schools</t>
+  </si>
+  <si>
+    <t>validUser</t>
+  </si>
+  <si>
+    <t>validPassword</t>
+  </si>
+  <si>
+    <t>Test@123</t>
+  </si>
+  <si>
+    <t>invalidUser</t>
+  </si>
+  <si>
+    <t>jkdbfbjdsbvi</t>
+  </si>
+  <si>
+    <t>invalidPassword</t>
+  </si>
+  <si>
+    <t>dhhdsuivb</t>
+  </si>
+  <si>
+    <t>space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>test@123</t>
+  </si>
+  <si>
+    <t>invalidUser1</t>
+  </si>
+  <si>
+    <t>40286@..09</t>
+  </si>
+  <si>
+    <t>invalidUser2</t>
+  </si>
+  <si>
+    <t>spaceUser</t>
+  </si>
+  <si>
+    <t>invalidOtp1</t>
+  </si>
+  <si>
+    <t>invalidOtp2</t>
+  </si>
+  <si>
+    <t>@@@@.....</t>
+  </si>
+  <si>
+    <t>validOtp</t>
+  </si>
+  <si>
+    <t>invalidPassword1</t>
+  </si>
+  <si>
+    <t>invalidPassword2</t>
+  </si>
+  <si>
+    <t>test123</t>
+  </si>
+  <si>
+    <t>Test@1234</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -67,13 +133,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,202 +472,202 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>title</v>
-      </c>
-      <c r="B2" t="str">
-        <v>EMIS | Tamil Nadu Schools</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>validUser</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
         <v>4028609</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>validPassword</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Test@123</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>invalidUser</v>
-      </c>
-      <c r="B5" t="str">
-        <v>jkdbfbjdsbvi</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>invalidPassword</v>
-      </c>
-      <c r="B6" t="str">
-        <v>dhhdsuivb</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>space</v>
-      </c>
-      <c r="B7" t="str">
-        <v xml:space="preserve">   </v>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>username</v>
-      </c>
-      <c r="B2" t="str">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2">
         <v>4028609</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>password</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Test@123</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>validUser</v>
-      </c>
-      <c r="B2" t="str">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
         <v>4028609</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>invalidUser1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>40286@..09</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>invalidUser2</v>
-      </c>
-      <c r="B4" t="str">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
         <v>4028609548494</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>spaceUser</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>invalidOtp1</v>
-      </c>
-      <c r="B6" t="str">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6">
         <v>8555555</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>invalidOtp2</v>
-      </c>
-      <c r="B7" t="str">
-        <v>@@@@.....</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>validOtp</v>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>invalidPassword1</v>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>invalidPassword2</v>
-      </c>
-      <c r="B10" t="str">
-        <v>test123</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>validPassword</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Test@1234</v>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
demo note added and files were modified
</commit_message>
<xml_diff>
--- a/data/excel/TestData.xlsx
+++ b/data/excel/TestData.xlsx
@@ -127,7 +127,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -135,16 +135,31 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8EAADA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3EFD9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -152,12 +167,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,83 +524,86 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
+    <col min="2" max="2" width="18.142857142857142" customWidth="1"/>
+    <col min="3" max="3" width="20.714285714285715" customWidth="1"/>
+    <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>4028609</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>4028619</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -591,329 +618,330 @@
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="5" width="14.714285714285714" customWidth="1"/>
+    <col min="6" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>30648666</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>30648666</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>4028619</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>4028619</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>4028611</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>4028621</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>20233863</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>20233863</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>1</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>2</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>4028612</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>4028622</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>2</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>3</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>4028613</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>4028623</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="A13" s="2">
         <v>3</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>1</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="2">
         <v>4028609</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="2">
         <v>4028619</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>1</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>2</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>4028614</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="2">
         <v>4028624</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>2</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="A18" s="2">
         <v>3</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>4028615</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="2">
         <v>4028625</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>3</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -928,109 +956,116 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="3" width="16.285714285714285" customWidth="1"/>
+    <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>4028609</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>4028609</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>4028609548494</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>4028609548494</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>8555555</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>8555555</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>